<commit_message>
Completed calculations on total insights
</commit_message>
<xml_diff>
--- a/bulky_upload_files/agents_template_test.xlsx
+++ b/bulky_upload_files/agents_template_test.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="41">
   <si>
     <t>first_name</t>
   </si>
@@ -138,6 +138,15 @@
   </si>
   <si>
     <t>phone_numberr</t>
+  </si>
+  <si>
+    <t>agent_type</t>
+  </si>
+  <si>
+    <t>VOICE_LVC</t>
+  </si>
+  <si>
+    <t>VOICE_HVC</t>
   </si>
 </sst>
 </file>
@@ -482,196 +491,205 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.21875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14.6640625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="16.33203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="9.88671875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="20.5546875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="14.77734375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="16.33203125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="13" style="1" customWidth="1"/>
-    <col min="10" max="10" width="12" style="1" customWidth="1"/>
-    <col min="11" max="11" width="22.44140625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="13.44140625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="21.6640625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="16.6640625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="15.21875" style="1" customWidth="1"/>
-    <col min="16" max="16" width="15.5546875" style="1" customWidth="1"/>
-    <col min="17" max="17" width="15.77734375" style="1" customWidth="1"/>
-    <col min="18" max="18" width="14.5546875" style="1" customWidth="1"/>
-    <col min="19" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="2" width="14.21875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="14.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="9.88671875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20.5546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="14.77734375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="16.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="13" style="1" customWidth="1"/>
+    <col min="11" max="11" width="12" style="1" customWidth="1"/>
+    <col min="12" max="12" width="22.44140625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="13.44140625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="21.6640625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="16.6640625" style="1" customWidth="1"/>
+    <col min="16" max="16" width="15.21875" style="1" customWidth="1"/>
+    <col min="17" max="17" width="15.5546875" style="1" customWidth="1"/>
+    <col min="18" max="18" width="15.77734375" style="1" customWidth="1"/>
+    <col min="19" max="19" width="14.5546875" style="1" customWidth="1"/>
+    <col min="20" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="2" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" s="2" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="1">
         <v>1</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="L2" s="4">
+      <c r="M2" s="4">
         <v>32909</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>20</v>
       </c>
       <c r="P2" s="1" t="s">
         <v>20</v>
       </c>
       <c r="Q2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="R2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="R2" s="1" t="s">
+      <c r="S2" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="1">
         <v>3</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="L3" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="L3" s="4">
+      <c r="M3" s="4">
         <v>25628</v>
       </c>
-      <c r="M3" s="1" t="s">
+      <c r="N3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="N3" s="1" t="s">
+      <c r="O3" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="O3" s="1" t="s">
-        <v>20</v>
       </c>
       <c r="P3" s="1" t="s">
         <v>20</v>
       </c>
       <c r="Q3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="R3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="R3" s="1" t="s">
+      <c r="S3" s="1" t="s">
         <v>30</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1"/>
-    <hyperlink ref="F3" r:id="rId2"/>
+    <hyperlink ref="G2" r:id="rId1"/>
+    <hyperlink ref="G3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId3"/>

</xml_diff>